<commit_message>
scan: seg0 2026-09-18 18:04 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-09-18.xlsx
+++ b/output/full_scan/batch_seq1_2026-09-18.xlsx
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>250.7454743954218</v>
+        <v>250.7454743954217</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>721</v>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>235.8916936432086</v>
+        <v>235.8916936432085</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>0</v>

</xml_diff>